<commit_message>
pre infinite loop, play again not being clicked
</commit_message>
<xml_diff>
--- a/src/wordle_log.xlsx
+++ b/src/wordle_log.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,12 +486,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -501,7 +501,7 @@
           <t>S</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>E</t>
         </is>
@@ -514,29 +514,29 @@
       <c r="B3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>E</t>
         </is>
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>D</t>
         </is>
       </c>
     </row>
@@ -547,227 +547,224 @@
       <c r="B4" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" t="n">
-        <v>2</v>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>JETTY</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="n">
         <v>2</v>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
           <t>O</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="9"/>
+    </row>
     <row r="10">
       <c r="A10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" t="n">
         <v>3</v>
       </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>U</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>T</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ABOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" t="n">
         <v>3</v>
       </c>
-      <c r="B11" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>3</v>
-      </c>
-      <c r="B12" t="n">
-        <v>3</v>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G13" s="1" t="inlineStr">
         <is>
           <t>E</t>
         </is>
@@ -775,98 +772,98 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>T</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>I</t>
         </is>
       </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>L</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>L</t>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" t="n">
         <v>4</v>
       </c>
-      <c r="B16" t="n">
-        <v>3</v>
-      </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>I</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="F16" s="1" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G16" s="1" t="inlineStr">
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>H</t>
         </is>
@@ -874,34 +871,541 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>FINCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" t="n">
         <v>4</v>
       </c>
-      <c r="B17" t="n">
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
         <v>4</v>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>PRONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>5</v>
+      </c>
+      <c r="B26" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>DINER</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>6</v>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>6</v>
+      </c>
+      <c r="B30" t="n">
+        <v>2</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>6</v>
+      </c>
+      <c r="B31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G31" s="1" t="inlineStr">
         <is>
           <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>6</v>
+      </c>
+      <c r="B32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>6</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>TRIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>7</v>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>7</v>
+      </c>
+      <c r="B36" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>7</v>
+      </c>
+      <c r="B37" t="n">
+        <v>3</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>7</v>
+      </c>
+      <c r="B38" t="n">
+        <v>4</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>7</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>EDICT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
infinite loop working perfectly. Next step Data logging and excel creation
</commit_message>
<xml_diff>
--- a/src/wordle_log.xlsx
+++ b/src/wordle_log.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G374"/>
+  <dimension ref="A1:G492"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9684,6 +9684,7 @@
         </is>
       </c>
     </row>
+    <row r="370"/>
     <row r="371">
       <c r="A371" t="n">
         <v>65</v>
@@ -9795,6 +9796,2871 @@
       <c r="C374" t="inlineStr">
         <is>
           <t>EAGLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="375"/>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>66</v>
+      </c>
+      <c r="B376" t="n">
+        <v>1</v>
+      </c>
+      <c r="C376" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D376" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E376" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F376" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G376" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="n">
+        <v>66</v>
+      </c>
+      <c r="B377" t="n">
+        <v>2</v>
+      </c>
+      <c r="C377" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D377" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E377" s="1" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F377" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="G377" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="n">
+        <v>66</v>
+      </c>
+      <c r="B378" t="n">
+        <v>3</v>
+      </c>
+      <c r="C378" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D378" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E378" s="1" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F378" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G378" s="1" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="n">
+        <v>66</v>
+      </c>
+      <c r="B379" t="n">
+        <v>4</v>
+      </c>
+      <c r="C379" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D379" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E379" s="3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F379" s="3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G379" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="n">
+        <v>66</v>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>TODDY</t>
+        </is>
+      </c>
+    </row>
+    <row r="381"/>
+    <row r="382">
+      <c r="A382" t="n">
+        <v>67</v>
+      </c>
+      <c r="B382" t="n">
+        <v>1</v>
+      </c>
+      <c r="C382" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D382" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E382" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F382" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G382" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="n">
+        <v>67</v>
+      </c>
+      <c r="B383" t="n">
+        <v>2</v>
+      </c>
+      <c r="C383" s="1" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="D383" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E383" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F383" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G383" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="n">
+        <v>67</v>
+      </c>
+      <c r="B384" t="n">
+        <v>3</v>
+      </c>
+      <c r="C384" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D384" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="E384" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F384" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G384" s="1" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="n">
+        <v>67</v>
+      </c>
+      <c r="B385" t="n">
+        <v>4</v>
+      </c>
+      <c r="C385" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D385" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="E385" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F385" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G385" s="1" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="n">
+        <v>67</v>
+      </c>
+      <c r="B386" t="n">
+        <v>5</v>
+      </c>
+      <c r="C386" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D386" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="E386" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F386" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G386" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="n">
+        <v>67</v>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>STINT</t>
+        </is>
+      </c>
+    </row>
+    <row r="388"/>
+    <row r="389">
+      <c r="A389" t="n">
+        <v>68</v>
+      </c>
+      <c r="B389" t="n">
+        <v>1</v>
+      </c>
+      <c r="C389" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D389" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E389" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F389" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G389" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="n">
+        <v>68</v>
+      </c>
+      <c r="B390" t="n">
+        <v>2</v>
+      </c>
+      <c r="C390" s="1" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="D390" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E390" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F390" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G390" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="391"/>
+    <row r="392">
+      <c r="A392" t="n">
+        <v>69</v>
+      </c>
+      <c r="B392" t="n">
+        <v>1</v>
+      </c>
+      <c r="C392" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D392" s="2" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E392" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F392" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G392" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="n">
+        <v>69</v>
+      </c>
+      <c r="B393" t="n">
+        <v>2</v>
+      </c>
+      <c r="C393" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D393" s="1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E393" s="1" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F393" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G393" s="2" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="n">
+        <v>69</v>
+      </c>
+      <c r="B394" t="n">
+        <v>3</v>
+      </c>
+      <c r="C394" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E394" s="1" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="F394" s="2" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G394" s="1" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="n">
+        <v>69</v>
+      </c>
+      <c r="B395" t="n">
+        <v>4</v>
+      </c>
+      <c r="C395" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D395" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="E395" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F395" s="3" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="G395" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="n">
+        <v>69</v>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>RERUN</t>
+        </is>
+      </c>
+    </row>
+    <row r="397"/>
+    <row r="398">
+      <c r="A398" t="n">
+        <v>70</v>
+      </c>
+      <c r="B398" t="n">
+        <v>1</v>
+      </c>
+      <c r="C398" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D398" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E398" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F398" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G398" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="n">
+        <v>70</v>
+      </c>
+      <c r="B399" t="n">
+        <v>2</v>
+      </c>
+      <c r="C399" s="2" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="D399" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E399" s="1" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="F399" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G399" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="n">
+        <v>70</v>
+      </c>
+      <c r="B400" t="n">
+        <v>3</v>
+      </c>
+      <c r="C400" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D400" s="2" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E400" s="1" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F400" s="1" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="G400" s="1" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="n">
+        <v>70</v>
+      </c>
+      <c r="B401" t="n">
+        <v>4</v>
+      </c>
+      <c r="C401" s="1" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D401" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E401" s="3" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F401" s="3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G401" s="3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="n">
+        <v>70</v>
+      </c>
+      <c r="B402" t="n">
+        <v>5</v>
+      </c>
+      <c r="C402" s="3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D402" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E402" s="3" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F402" s="3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G402" s="3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="n">
+        <v>70</v>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>FLUFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="404"/>
+    <row r="405">
+      <c r="A405" t="n">
+        <v>71</v>
+      </c>
+      <c r="B405" t="n">
+        <v>1</v>
+      </c>
+      <c r="C405" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D405" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E405" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F405" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G405" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="406"/>
+    <row r="407">
+      <c r="A407" t="n">
+        <v>72</v>
+      </c>
+      <c r="B407" t="n">
+        <v>1</v>
+      </c>
+      <c r="C407" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D407" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E407" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F407" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G407" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="n">
+        <v>72</v>
+      </c>
+      <c r="B408" t="n">
+        <v>2</v>
+      </c>
+      <c r="C408" s="1" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D408" s="2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E408" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F408" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G408" s="1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="n">
+        <v>72</v>
+      </c>
+      <c r="B409" t="n">
+        <v>3</v>
+      </c>
+      <c r="C409" s="3" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D409" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="E409" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F409" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G409" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="n">
+        <v>72</v>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>HELIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="411"/>
+    <row r="412">
+      <c r="A412" t="n">
+        <v>73</v>
+      </c>
+      <c r="B412" t="n">
+        <v>1</v>
+      </c>
+      <c r="C412" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D412" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E412" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F412" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G412" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="n">
+        <v>73</v>
+      </c>
+      <c r="B413" t="n">
+        <v>2</v>
+      </c>
+      <c r="C413" s="1" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D413" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E413" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F413" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G413" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="n">
+        <v>73</v>
+      </c>
+      <c r="B414" t="n">
+        <v>3</v>
+      </c>
+      <c r="C414" s="1" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D414" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E414" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F414" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G414" s="1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="n">
+        <v>73</v>
+      </c>
+      <c r="B415" t="n">
+        <v>4</v>
+      </c>
+      <c r="C415" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D415" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E415" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F415" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G415" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="n">
+        <v>73</v>
+      </c>
+      <c r="B416" t="n">
+        <v>5</v>
+      </c>
+      <c r="C416" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D416" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E416" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F416" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G416" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="n">
+        <v>73</v>
+      </c>
+      <c r="B417" t="n">
+        <v>6</v>
+      </c>
+      <c r="C417" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D417" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E417" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F417" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G417" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="n">
+        <v>73</v>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>GRAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="419"/>
+    <row r="420">
+      <c r="A420" t="n">
+        <v>74</v>
+      </c>
+      <c r="B420" t="n">
+        <v>1</v>
+      </c>
+      <c r="C420" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D420" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E420" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F420" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G420" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="421"/>
+    <row r="422">
+      <c r="A422" t="n">
+        <v>75</v>
+      </c>
+      <c r="B422" t="n">
+        <v>1</v>
+      </c>
+      <c r="C422" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D422" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E422" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F422" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G422" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="n">
+        <v>75</v>
+      </c>
+      <c r="B423" t="n">
+        <v>2</v>
+      </c>
+      <c r="C423" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D423" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E423" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F423" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="G423" s="1" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="n">
+        <v>75</v>
+      </c>
+      <c r="B424" t="n">
+        <v>3</v>
+      </c>
+      <c r="C424" s="1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D424" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E424" s="3" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F424" s="3" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G424" s="3" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="n">
+        <v>75</v>
+      </c>
+      <c r="B425" t="n">
+        <v>4</v>
+      </c>
+      <c r="C425" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D425" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E425" s="3" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F425" s="3" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G425" s="3" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="n">
+        <v>75</v>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>BOUGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="427"/>
+    <row r="428">
+      <c r="A428" t="n">
+        <v>76</v>
+      </c>
+      <c r="B428" t="n">
+        <v>1</v>
+      </c>
+      <c r="C428" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D428" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E428" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F428" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G428" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="n">
+        <v>76</v>
+      </c>
+      <c r="B429" t="n">
+        <v>2</v>
+      </c>
+      <c r="C429" s="1" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D429" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E429" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F429" s="1" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G429" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="n">
+        <v>76</v>
+      </c>
+      <c r="B430" t="n">
+        <v>3</v>
+      </c>
+      <c r="C430" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D430" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E430" s="1" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F430" s="1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G430" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="n">
+        <v>76</v>
+      </c>
+      <c r="B431" t="n">
+        <v>4</v>
+      </c>
+      <c r="C431" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D431" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E431" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F431" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G431" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="n">
+        <v>76</v>
+      </c>
+      <c r="B432" t="n">
+        <v>5</v>
+      </c>
+      <c r="C432" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D432" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E432" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F432" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G432" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="n">
+        <v>76</v>
+      </c>
+      <c r="B433" t="n">
+        <v>6</v>
+      </c>
+      <c r="C433" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D433" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E433" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F433" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G433" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="n">
+        <v>76</v>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>CREME</t>
+        </is>
+      </c>
+    </row>
+    <row r="435"/>
+    <row r="436">
+      <c r="A436" t="n">
+        <v>77</v>
+      </c>
+      <c r="B436" t="n">
+        <v>1</v>
+      </c>
+      <c r="C436" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D436" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E436" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F436" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G436" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="n">
+        <v>77</v>
+      </c>
+      <c r="B437" t="n">
+        <v>2</v>
+      </c>
+      <c r="C437" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D437" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E437" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F437" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G437" s="1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="n">
+        <v>77</v>
+      </c>
+      <c r="B438" t="n">
+        <v>3</v>
+      </c>
+      <c r="C438" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D438" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E438" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F438" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G438" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="n">
+        <v>77</v>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>ALLEY</t>
+        </is>
+      </c>
+    </row>
+    <row r="440"/>
+    <row r="441">
+      <c r="A441" t="n">
+        <v>78</v>
+      </c>
+      <c r="B441" t="n">
+        <v>1</v>
+      </c>
+      <c r="C441" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D441" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E441" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F441" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G441" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="n">
+        <v>78</v>
+      </c>
+      <c r="B442" t="n">
+        <v>2</v>
+      </c>
+      <c r="C442" s="1" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D442" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E442" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F442" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G442" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="n">
+        <v>78</v>
+      </c>
+      <c r="B443" t="n">
+        <v>3</v>
+      </c>
+      <c r="C443" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D443" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E443" s="1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F443" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G443" s="1" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="n">
+        <v>78</v>
+      </c>
+      <c r="B444" t="n">
+        <v>4</v>
+      </c>
+      <c r="C444" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D444" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E444" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F444" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G444" s="3" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="n">
+        <v>78</v>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>TOPAZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="446"/>
+    <row r="447">
+      <c r="A447" t="n">
+        <v>79</v>
+      </c>
+      <c r="B447" t="n">
+        <v>1</v>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="448"/>
+    <row r="449">
+      <c r="A449" t="n">
+        <v>80</v>
+      </c>
+      <c r="B449" t="n">
+        <v>1</v>
+      </c>
+      <c r="C449" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D449" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E449" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F449" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G449" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="n">
+        <v>80</v>
+      </c>
+      <c r="B450" t="n">
+        <v>2</v>
+      </c>
+      <c r="C450" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D450" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="E450" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F450" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G450" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="n">
+        <v>80</v>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>LEAST</t>
+        </is>
+      </c>
+    </row>
+    <row r="452"/>
+    <row r="453">
+      <c r="A453" t="n">
+        <v>81</v>
+      </c>
+      <c r="B453" t="n">
+        <v>1</v>
+      </c>
+      <c r="C453" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D453" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E453" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F453" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G453" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="n">
+        <v>81</v>
+      </c>
+      <c r="B454" t="n">
+        <v>2</v>
+      </c>
+      <c r="C454" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D454" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E454" s="1" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F454" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G454" s="1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="n">
+        <v>81</v>
+      </c>
+      <c r="B455" t="n">
+        <v>3</v>
+      </c>
+      <c r="C455" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D455" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E455" s="1" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F455" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G455" s="1" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="n">
+        <v>81</v>
+      </c>
+      <c r="B456" t="n">
+        <v>4</v>
+      </c>
+      <c r="C456" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D456" s="1" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="E456" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="F456" s="1" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G456" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="n">
+        <v>81</v>
+      </c>
+      <c r="B457" t="n">
+        <v>5</v>
+      </c>
+      <c r="C457" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D457" s="3" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="E457" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="F457" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G457" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="n">
+        <v>81</v>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>EVENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="459"/>
+    <row r="460">
+      <c r="A460" t="n">
+        <v>82</v>
+      </c>
+      <c r="B460" t="n">
+        <v>1</v>
+      </c>
+      <c r="C460" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D460" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E460" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F460" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G460" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="n">
+        <v>82</v>
+      </c>
+      <c r="B461" t="n">
+        <v>2</v>
+      </c>
+      <c r="C461" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D461" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E461" s="1" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F461" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G461" s="1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="n">
+        <v>82</v>
+      </c>
+      <c r="B462" t="n">
+        <v>3</v>
+      </c>
+      <c r="C462" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D462" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="E462" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F462" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G462" s="3" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="n">
+        <v>82</v>
+      </c>
+      <c r="B463" t="n">
+        <v>4</v>
+      </c>
+      <c r="C463" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D463" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="E463" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="F463" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G463" s="3" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="n">
+        <v>82</v>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>TEETH</t>
+        </is>
+      </c>
+    </row>
+    <row r="465"/>
+    <row r="466">
+      <c r="A466" t="n">
+        <v>83</v>
+      </c>
+      <c r="B466" t="n">
+        <v>1</v>
+      </c>
+      <c r="C466" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D466" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E466" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F466" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G466" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="n">
+        <v>83</v>
+      </c>
+      <c r="B467" t="n">
+        <v>2</v>
+      </c>
+      <c r="C467" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D467" s="1" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E467" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F467" s="1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G467" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="n">
+        <v>83</v>
+      </c>
+      <c r="B468" t="n">
+        <v>3</v>
+      </c>
+      <c r="C468" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D468" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E468" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F468" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G468" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="n">
+        <v>83</v>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>ASSAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="470"/>
+    <row r="471">
+      <c r="A471" t="n">
+        <v>84</v>
+      </c>
+      <c r="B471" t="n">
+        <v>1</v>
+      </c>
+      <c r="C471" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D471" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E471" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F471" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G471" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="n">
+        <v>84</v>
+      </c>
+      <c r="B472" t="n">
+        <v>2</v>
+      </c>
+      <c r="C472" s="1" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D472" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E472" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F472" s="1" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G472" s="1" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="n">
+        <v>84</v>
+      </c>
+      <c r="B473" t="n">
+        <v>3</v>
+      </c>
+      <c r="C473" s="1" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D473" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E473" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F473" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G473" s="1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="n">
+        <v>84</v>
+      </c>
+      <c r="B474" t="n">
+        <v>4</v>
+      </c>
+      <c r="C474" s="3" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D474" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E474" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F474" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="G474" s="3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="n">
+        <v>84</v>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>GLOOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="476"/>
+    <row r="477">
+      <c r="A477" t="n">
+        <v>85</v>
+      </c>
+      <c r="B477" t="n">
+        <v>1</v>
+      </c>
+      <c r="C477" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D477" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E477" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F477" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G477" s="1" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="n">
+        <v>85</v>
+      </c>
+      <c r="B478" t="n">
+        <v>2</v>
+      </c>
+      <c r="C478" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D478" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E478" s="1" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F478" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="G478" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="n">
+        <v>85</v>
+      </c>
+      <c r="B479" t="n">
+        <v>3</v>
+      </c>
+      <c r="C479" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D479" s="3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E479" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F479" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="G479" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="n">
+        <v>85</v>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>IDIOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="481"/>
+    <row r="482">
+      <c r="A482" t="n">
+        <v>86</v>
+      </c>
+      <c r="B482" t="n">
+        <v>1</v>
+      </c>
+      <c r="C482" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D482" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E482" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F482" s="1" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G482" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="n">
+        <v>86</v>
+      </c>
+      <c r="B483" t="n">
+        <v>2</v>
+      </c>
+      <c r="C483" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="D483" s="1" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E483" s="3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F483" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G483" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="n">
+        <v>86</v>
+      </c>
+      <c r="B484" t="n">
+        <v>3</v>
+      </c>
+      <c r="C484" s="1" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D484" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E484" s="3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F484" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G484" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="n">
+        <v>86</v>
+      </c>
+      <c r="B485" t="n">
+        <v>4</v>
+      </c>
+      <c r="C485" s="1" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D485" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E485" s="3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F485" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G485" s="1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="n">
+        <v>86</v>
+      </c>
+      <c r="B486" t="n">
+        <v>5</v>
+      </c>
+      <c r="C486" s="3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D486" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E486" s="3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F486" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G486" s="3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="n">
+        <v>86</v>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>MODEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="n">
+        <v>87</v>
+      </c>
+      <c r="B489" t="n">
+        <v>1</v>
+      </c>
+      <c r="C489" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D489" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E489" s="1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F489" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G489" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="n">
+        <v>87</v>
+      </c>
+      <c r="B490" t="n">
+        <v>2</v>
+      </c>
+      <c r="C490" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D490" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E490" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F490" s="1" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G490" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="n">
+        <v>87</v>
+      </c>
+      <c r="B491" t="n">
+        <v>3</v>
+      </c>
+      <c r="C491" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D491" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E491" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F491" s="3" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="G491" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="n">
+        <v>87</v>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>ENSUE</t>
         </is>
       </c>
     </row>

</xml_diff>